<commit_message>
ATENÇÃO FASE 2 - REFATORADO SCRIPTS
</commit_message>
<xml_diff>
--- a/projetos/OBRA_TMULT/04_PRODUCAO_E_AVANCO/MATRIZ_BLOQUEIO_FVS_CONTRATOS_TMULT.xlsx
+++ b/projetos/OBRA_TMULT/04_PRODUCAO_E_AVANCO/MATRIZ_BLOQUEIO_FVS_CONTRATOS_TMULT.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,7 +29,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="13"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -47,26 +47,16 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001B365D"/>
-      <sz val="9"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00C5221F"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00137333"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="9"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -97,14 +87,8 @@
         <bgColor rgb="00F8F9FA"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E6F4EA"/>
-        <bgColor rgb="00E6F4EA"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -126,37 +110,23 @@
         <color rgb="00DDDDDD"/>
       </bottom>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00E0E0E0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00E0E0E0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00E0E0E0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00E0E0E0"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -164,24 +134,15 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -548,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -558,8 +519,6 @@
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -612,16 +571,6 @@
           <t>Serviço Sucessor Condicionado</t>
         </is>
       </c>
-      <c r="H3" s="13" t="inlineStr">
-        <is>
-          <t>Status Atual de Campo</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="inlineStr">
-        <is>
-          <t>Última Inspeção</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -694,16 +643,6 @@
       <c r="G5" s="12" t="inlineStr">
         <is>
           <t>Lançamento de concreto estrutural usinado e reaterro de valas</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="inlineStr">
-        <is>
-          <t>🟢 Aprovado</t>
-        </is>
-      </c>
-      <c r="I5" s="15" t="inlineStr">
-        <is>
-          <t>29/09/2026</t>
         </is>
       </c>
     </row>

</xml_diff>